<commit_message>
Enhance com_eqa: thêm "Năm bắt đầu sử dụng" vào thông tin quản lý môn học
</commit_message>
<xml_diff>
--- a/media/com_eqa/xlsx/sample_subjects.xlsx
+++ b/media/com_eqa/xlsx/sample_subjects.xlsx
@@ -1,182 +1,169 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Departerment Website\Claude Cowork\TEMPORARY FILES\subject-start-year\com_eqa\media\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62CC67F-F8F2-4363-A728-DA41F6583E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681A5903-1AA7-4711-BFEF-7D9075DBACF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B762B903-6094-4588-AAE4-7206B1850746}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$C$15</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
+  <si>
+    <t>Khoa</t>
+  </si>
   <si>
     <t>Mã HP</t>
   </si>
   <si>
+    <t>Môn học</t>
+  </si>
+  <si>
+    <t>Bậc học</t>
+  </si>
+  <si>
     <t>Số TC</t>
   </si>
   <si>
+    <t>Hình thức thi</t>
+  </si>
+  <si>
+    <t>Ngân hàng</t>
+  </si>
+  <si>
+    <t>Năm SD</t>
+  </si>
+  <si>
+    <t>KAT</t>
+  </si>
+  <si>
+    <t>ATAT1</t>
+  </si>
+  <si>
+    <t>An toàn mạng máy tính</t>
+  </si>
+  <si>
+    <t>ĐH</t>
+  </si>
+  <si>
+    <t>Tự luận</t>
+  </si>
+  <si>
+    <t>KCN</t>
+  </si>
+  <si>
+    <t>ATCTHT5</t>
+  </si>
+  <si>
+    <t>Bộ giao thức TCP/IP và định tuyến mạng</t>
+  </si>
+  <si>
+    <t>Thực hành</t>
+  </si>
+  <si>
+    <t>KDV</t>
+  </si>
+  <si>
+    <t>F9</t>
+  </si>
+  <si>
+    <t>Cấu kiện điện tử</t>
+  </si>
+  <si>
+    <t>Trắc nghiệm</t>
+  </si>
+  <si>
+    <t>CKCTKM1</t>
+  </si>
+  <si>
+    <t>Cấu trúc Dữ liệu và giải thuật</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>Cơ sở lý thuyết truyền tin</t>
+  </si>
+  <si>
+    <t>KMM</t>
+  </si>
+  <si>
+    <t>MMNV1</t>
+  </si>
+  <si>
+    <t>Chính trị nghiệp vụ</t>
+  </si>
+  <si>
+    <t>F19</t>
+  </si>
+  <si>
+    <t>Điện tử số - Vi xử lý</t>
+  </si>
+  <si>
     <t>HMDVKV1</t>
   </si>
   <si>
-    <t>ATAT1</t>
+    <t>Điện tử số</t>
   </si>
   <si>
     <t>CTKT12</t>
   </si>
   <si>
+    <t>Đồ án môn học 2. Thực tập về Phát  triển Web</t>
+  </si>
+  <si>
+    <t>Đồ án</t>
+  </si>
+  <si>
+    <t>KCB</t>
+  </si>
+  <si>
+    <t>CBTT2.1</t>
+  </si>
+  <si>
+    <t>Giải tích 2</t>
+  </si>
+  <si>
+    <t>KQG</t>
+  </si>
+  <si>
+    <t>HMQGTC23</t>
+  </si>
+  <si>
+    <t>Giáo dục thể chất 2</t>
+  </si>
+  <si>
+    <t>HMQGTC3</t>
+  </si>
+  <si>
+    <t>Giáo dục thể chất 3</t>
+  </si>
+  <si>
+    <t>HMQGTC4</t>
+  </si>
+  <si>
+    <t>Giáo dục thể chất 4</t>
+  </si>
+  <si>
     <t>HMQGTC5</t>
   </si>
   <si>
-    <t>ATCTHT5</t>
-  </si>
-  <si>
-    <t>HMQGTC3</t>
-  </si>
-  <si>
-    <t>HMQGTC4</t>
-  </si>
-  <si>
-    <t>MMNV1</t>
-  </si>
-  <si>
-    <t>CBTT2.1</t>
-  </si>
-  <si>
-    <t>CKCTKM1</t>
-  </si>
-  <si>
-    <t>F19</t>
-  </si>
-  <si>
-    <t>F6</t>
-  </si>
-  <si>
-    <t>Điện tử số - Vi xử lý</t>
-  </si>
-  <si>
-    <t>Cơ sở lý thuyết truyền tin</t>
-  </si>
-  <si>
-    <t>F9</t>
-  </si>
-  <si>
-    <t>Cấu kiện điện tử</t>
-  </si>
-  <si>
-    <t>An toàn mạng máy tính</t>
-  </si>
-  <si>
-    <t>Môn học</t>
-  </si>
-  <si>
-    <t>Bộ giao thức TCP/IP và định tuyến mạng</t>
-  </si>
-  <si>
-    <t>Cấu trúc Dữ liệu và giải thuật</t>
-  </si>
-  <si>
-    <t>Chính trị nghiệp vụ</t>
-  </si>
-  <si>
-    <t>Điện tử số</t>
-  </si>
-  <si>
-    <t>Đồ án môn học 2. Thực tập về Phát  triển Web</t>
-  </si>
-  <si>
-    <t>Giáo dục thể chất 2</t>
-  </si>
-  <si>
-    <t>Giải tích 2</t>
-  </si>
-  <si>
-    <t>Giáo dục thể chất 3</t>
-  </si>
-  <si>
-    <t>Giáo dục thể chất 4</t>
-  </si>
-  <si>
     <t>Giáo dục thể chất 5</t>
-  </si>
-  <si>
-    <t>Hình thức thi</t>
-  </si>
-  <si>
-    <t>Tự luận</t>
-  </si>
-  <si>
-    <t>Trắc nghiệm</t>
-  </si>
-  <si>
-    <t>Thực hành</t>
-  </si>
-  <si>
-    <t>Ngân hàng</t>
-  </si>
-  <si>
-    <t>Khoa</t>
-  </si>
-  <si>
-    <t>KAT</t>
-  </si>
-  <si>
-    <t>KCN</t>
-  </si>
-  <si>
-    <t>KDV</t>
-  </si>
-  <si>
-    <t>KMM</t>
-  </si>
-  <si>
-    <t>KCB</t>
-  </si>
-  <si>
-    <t>KQG</t>
-  </si>
-  <si>
-    <t>Bậc học</t>
-  </si>
-  <si>
-    <t>ĐH</t>
-  </si>
-  <si>
-    <t>Đồ án</t>
-  </si>
-  <si>
-    <t>HMQGTC23</t>
   </si>
 </sst>
 </file>
@@ -605,375 +592,389 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A29353F-6DA1-41AC-88AB-D32A01CD9FD5}">
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.6328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="19" style="1" customWidth="1"/>
     <col min="3" max="3" width="58" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.6640625" style="1"/>
+    <col min="4" max="4" width="13.1796875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.6328125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E2" s="7">
         <v>3</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="G2" s="6">
         <v>2020</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H2" s="6">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E3" s="7">
         <v>3</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G3" s="6">
         <v>2017</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E4" s="7">
         <v>2</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G4" s="6">
         <v>2021</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H4" s="6">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E5" s="7">
         <v>3</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="G5" s="6">
         <v>2019</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H5" s="6">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="5" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E6" s="7">
         <v>2</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H6" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="5" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E7" s="7">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="5" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E8" s="7">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="D9" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E9" s="7">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>4</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E10" s="7">
         <v>3</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H10" s="6">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E11" s="7">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="G11" s="6">
         <v>2024</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E12" s="7">
         <v>1</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H12" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="C13" s="5" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E13" s="7">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G13" s="6"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H13" s="6">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E14" s="7">
         <v>1</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E15" s="7">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G15" s="6"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="7">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" s="6"/>
+      <c r="H15" s="6">
+        <v>2018</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:C16" xr:uid="{8A29353F-6DA1-41AC-88AB-D32A01CD9FD5}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C16">
-    <sortCondition ref="C2:C16"/>
-  </sortState>
-  <conditionalFormatting sqref="B2:B16">
-    <cfRule type="duplicateValues" dxfId="0" priority="34"/>
+  <autoFilter ref="B1:C15" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="B2:B15">
+    <cfRule type="duplicateValues" dxfId="0" priority="35"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>